<commit_message>
add: lua script engine
</commit_message>
<xml_diff>
--- a/config/配置_v2.0.xlsx
+++ b/config/配置_v2.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="18519" windowHeight="11218"/>
+    <workbookView windowWidth="18569" windowHeight="10825" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="project" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="83">
   <si>
     <t>key</t>
   </si>
@@ -253,27 +253,6 @@
   </si>
   <si>
     <t>127.0.0.1</t>
-  </si>
-  <si>
-    <t>ModbusRTU</t>
-  </si>
-  <si>
-    <t>/dev/ttyXRUSB2</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>/dev/ttyXRUSB3</t>
-  </si>
-  <si>
-    <t>/dev/ttyXRUSB1</t>
-  </si>
-  <si>
-    <t>/dev/ttyXRUSB4</t>
-  </si>
-  <si>
-    <t>/dev/ttyXRUSB5</t>
   </si>
   <si>
     <t>device_id</t>
@@ -1948,11 +1927,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="22.4017094017094" defaultRowHeight="18" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="22.4047619047619" defaultRowHeight="18" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="22.4017094017094" style="3"/>
-    <col min="2" max="2" width="33.7948717948718" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="22.4017094017094" style="3"/>
+    <col min="1" max="1" width="22.4047619047619" style="3"/>
+    <col min="2" max="2" width="33.7936507936508" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="22.4047619047619" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2122,8 +2101,8 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelRow="7" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="6.46153846153846" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.9316239316239" style="3" customWidth="1"/>
+    <col min="1" max="1" width="6.46031746031746" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.9285714285714" style="3" customWidth="1"/>
     <col min="3" max="3" width="20.3333333333333" style="3" customWidth="1"/>
     <col min="4" max="16384" width="9" style="3"/>
   </cols>
@@ -2230,18 +2209,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:Q8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelRow="7"/>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelRow="2"/>
   <cols>
-    <col min="1" max="1" width="6.46153846153846" style="3" customWidth="1"/>
-    <col min="2" max="2" width="15.5982905982906" style="3" customWidth="1"/>
-    <col min="3" max="3" width="13.4615384615385" style="3" customWidth="1"/>
-    <col min="4" max="4" width="12.9316239316239" style="3" customWidth="1"/>
-    <col min="5" max="5" width="44.5299145299145" style="3" customWidth="1"/>
-    <col min="6" max="10" width="12.1965811965812" style="3" customWidth="1"/>
+    <col min="1" max="1" width="6.46031746031746" style="3" customWidth="1"/>
+    <col min="2" max="2" width="15.5952380952381" style="3" customWidth="1"/>
+    <col min="3" max="3" width="13.4603174603175" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12.9285714285714" style="3" customWidth="1"/>
+    <col min="5" max="5" width="44.531746031746" style="3" customWidth="1"/>
+    <col min="6" max="10" width="12.1984126984127" style="3" customWidth="1"/>
     <col min="11" max="11" width="16.6666666666667" style="3" customWidth="1"/>
-    <col min="12" max="16" width="12.1965811965812" style="3" customWidth="1"/>
-    <col min="17" max="16384" width="9.06837606837607" style="3"/>
+    <col min="12" max="16" width="12.1984126984127" style="3" customWidth="1"/>
+    <col min="17" max="16384" width="9.07142857142857" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1" spans="1:17">
@@ -2318,7 +2297,7 @@
         <v>1000</v>
       </c>
       <c r="G2" s="3">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="L2" s="3">
         <v>500000</v>
@@ -2345,10 +2324,10 @@
         <v>71</v>
       </c>
       <c r="F3" s="3">
+        <v>2000</v>
+      </c>
+      <c r="G3" s="3">
         <v>1000</v>
-      </c>
-      <c r="G3" s="3">
-        <v>500</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>72</v>
@@ -2357,201 +2336,6 @@
         <v>33434</v>
       </c>
       <c r="J3" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17">
-      <c r="A4" s="3">
-        <f>devices!A4</f>
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G4" s="3">
-        <v>500</v>
-      </c>
-      <c r="J4" s="3">
-        <v>1</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" s="3">
-        <v>9600</v>
-      </c>
-      <c r="M4" s="3">
-        <v>8</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="O4" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17">
-      <c r="A5" s="3">
-        <f>devices!A5</f>
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G5" s="3">
-        <v>500</v>
-      </c>
-      <c r="J5" s="3">
-        <v>1</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="L5" s="3">
-        <v>9600</v>
-      </c>
-      <c r="M5" s="3">
-        <v>8</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="O5" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="3">
-        <f>devices!A6</f>
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G6" s="3">
-        <v>500</v>
-      </c>
-      <c r="J6" s="3">
-        <v>1</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="L6" s="3">
-        <v>9600</v>
-      </c>
-      <c r="M6" s="3">
-        <v>8</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="O6" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17">
-      <c r="A7" s="3">
-        <f>devices!A7</f>
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G7" s="3">
-        <v>500</v>
-      </c>
-      <c r="J7" s="3">
-        <v>1</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" s="3">
-        <v>9600</v>
-      </c>
-      <c r="M7" s="3">
-        <v>8</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="O7" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17">
-      <c r="A8" s="3">
-        <f>devices!A8</f>
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="3">
-        <v>500</v>
-      </c>
-      <c r="J8" s="3">
-        <v>1</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="L8" s="3">
-        <v>9600</v>
-      </c>
-      <c r="M8" s="3">
-        <v>8</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="O8" s="3">
         <v>1</v>
       </c>
     </row>
@@ -2568,27 +2352,27 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultColWidth="9.11111111111111" defaultRowHeight="18" outlineLevelRow="5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="11.7606837606838" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.6752136752137" style="2" customWidth="1"/>
-    <col min="3" max="3" width="144.854700854701" style="2" customWidth="1"/>
-    <col min="4" max="4" width="20.3931623931624" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.2905982905983" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.4358974358974" style="2" customWidth="1"/>
+    <col min="1" max="1" width="11.7619047619048" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.6746031746032" style="2" customWidth="1"/>
+    <col min="3" max="3" width="144.857142857143" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.3968253968254" style="2" customWidth="1"/>
+    <col min="5" max="5" width="10.2936507936508" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.4365079365079" style="2" customWidth="1"/>
     <col min="7" max="16384" width="9.11111111111111" style="2"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2599,7 +2383,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C2" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[2]遥测!$A$58:$A$71)</f>
@@ -2614,7 +2398,7 @@
         <v>44</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C3" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[2]遥测!$A$2:$A$55)</f>
@@ -2629,7 +2413,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C4" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥调!$A$2:$A$1000)</f>
@@ -2644,7 +2428,7 @@
         <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C5" s="2" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,[1]遥控!$A$2:$A$1000)</f>
@@ -2659,10 +2443,10 @@
         <v>42</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D6" s="2">
         <v>1</v>

</xml_diff>